<commit_message>
fix: normalize article codes by removing trailing # character
Parser now removes # character from article codes (e.g. CE20A# → CE20A),
preventing extraction of duplicate articles with identical quantities.

Result: Oferta 1 reduced from 1621 to 1510 articles (eliminated 111 duplicates).
Neconformitati reduced from 547 to 434 (eliminated 120 false EXTRA articles).
</commit_message>
<xml_diff>
--- a/output_AO/Raport_Oferta_2.xlsx
+++ b/output_AO/Raport_Oferta_2.xlsx
@@ -1113,8 +1113,8 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>IZD03D1  ton  12.0
-VOPSIRE CU VOPS MINIU CU APARAT AER COMPR 1 STR PECONF SI CTII METAL EXEC DIN PROF GROS 8-12 MM A material: manopera: utilaj: transport:</t>
+          <t>IZD04D1  tona  12.0
+VOPSIRE CU APARAT AER COMPR VOPSEA ULEI PE CONF SICONSTR MET PROFILE 8-12MM 2STRATURI material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
@@ -1134,8 +1134,8 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>IZD04D1  tona  12.0
-VOPSIRE CU APARAT AER COMPR VOPSEA ULEI PE CONF SICONSTR MET PROFILE 8-12MM 2STRATURI material: manopera: utilaj: transport:</t>
+          <t>IZD03D1  ton  12.0
+VOPSIRE CU VOPS MINIU CU APARAT AER COMPR 1 STR PECONF SI CTII METAL EXEC DIN PROF GROS 8-12 MM A material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
@@ -1737,8 +1737,8 @@
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>IZD03D1  tona  0.95
-VOPSIRE CU VOPS MINIU CU APARAT AER COMPR 1 STR PECONF SI CTII METAL EXEC DIN PROF GROS 8-12 MM material: manopera: utilaj: transport:</t>
+          <t>CB13I1  mp  300.0
+COFRAJE DIN PANOURI REFOLOSIBILE LA CONSTRUCTII CU H&lt;20M LA PLACI SI GRINZI CU PLACAJ DE 15MM material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
@@ -1758,8 +1758,8 @@
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>CB13I1  mp  300.0
-COFRAJE DIN PANOURI REFOLOSIBILE LA CONSTRUCTII CU H&lt;20M LA PLACI SI GRINZI CU PLACAJ DE 15MM material: manopera: utilaj: transport:</t>
+          <t>IZD03D1  tona  0.95
+VOPSIRE CU VOPS MINIU CU APARAT AER COMPR 1 STR PECONF SI CTII METAL EXEC DIN PROF GROS 8-12 MM material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -1804,13 +1804,13 @@
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>CK23A#  mp  6.0
+          <t>CK23A  mp  6.0
 Ferestre din mase plastice cu unul sau mai multe canaturi, supraf toc mai mare 1.00 mp, la ctii cu H mai mic sau egal 35 m</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>CK23A#  m  6.0
+          <t>CK23A  m  6.0
 Ferestre din mase plastice cu unul sau mai multe canaturi, supraf toc mai mare 1.00 mp, la ctii cu H mai mic sau egal mp material: manopera: utilaj: transport:</t>
         </is>
       </c>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>CF15C#  mp  408.0
+          <t>CF15C  mp  408.0
 Tencuieli interioare finisaj fin sclivisite,de 0.5 cm grosime, la pereti din beton cu suprafete plane, executate manual, cu mortar DESIGN STUDIO S.R.L. - proiect inițial 424/2018 · proiect actualizat integral 424-rev/ 2024</t>
         </is>
       </c>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>CI06C#  mp  213.0
+          <t>CI06C  mp  213.0
 Placaj faianta, aceeasi culoare si format, 15 cm-30x30 cm, fixate cu aditiv, pe supr plane pereti si stalpi</t>
         </is>
       </c>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="B110" s="8" t="inlineStr">
         <is>
-          <t>SA14B#  ml  70.0
+          <t>SA14B  ml  70.0
 TEAVA MAT PL (PP, PE, PP-R) IMBINARE PRIN SUDURA PRIN POLIFUZIUNE, LA CTII IND, D=20 MM</t>
         </is>
       </c>
@@ -2844,7 +2844,7 @@
       </c>
       <c r="B116" s="8" t="inlineStr">
         <is>
-          <t>SA14C#  m  75.0
+          <t>SA14C  m  75.0
 TEAVA MAT PL (PP, PE, PP-R) IMBINATA PRIN SUDURA PRIN POLIFUZIUNE, LA CTII IND. , D= 25 MM 424-rev/ 2024 DESIGN STUDIO S.R.L. - proiect inițial 424/2018 - proiect actualizat integral</t>
         </is>
       </c>
@@ -5916,13 +5916,13 @@
       </c>
       <c r="B265" s="8" t="inlineStr">
         <is>
-          <t>CK23A#  mp  26.0
+          <t>CK23A  mp  26.0
 Ferestre din mase plastice cu unul sau mai multe canaturi, supraf toc mai mare 1.00 mp, la ctii cu H mai mic sau egal 35 m</t>
         </is>
       </c>
       <c r="C265" s="8" t="inlineStr">
         <is>
-          <t>CK23A#  m  26.0
+          <t>CK23A  m  26.0
 Ferestre din mase plastice cu unul sau mai multe canaturi, supraf toc mai mare 1.00 mp, la ctii cu H mai mic sau egal mp material: manopera: utilaj: transport: 27.L FERESTRE DIN PROFILE PVC CU GEAM TERMOIZOLANT MP.</t>
         </is>
       </c>
@@ -6044,7 +6044,7 @@
       </c>
       <c r="B271" s="8" t="inlineStr">
         <is>
-          <t>CF15C#  mp  873.0
+          <t>CF15C  mp  873.0
 Tencuieli interioare finisaj fin sclivisite, de 0.5 cm grosime, la pereti din beton cu suprafete plane, executate manual, cu mortar DESIGN STUDIO S.R.L. - proiect inițial 424/2018 - proiect actualizat integral 424-rev/ 2024</t>
         </is>
       </c>
@@ -6086,7 +6086,7 @@
       </c>
       <c r="B273" s="8" t="inlineStr">
         <is>
-          <t>CI06C#  mp  282.0
+          <t>CI06C  mp  282.0
 Placaj faianta, aceeasi culoare si format, 15 cm-30x30 cm, fixate cu aditiv, pe supr plane pereti si stalpi</t>
         </is>
       </c>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="B323" s="8" t="inlineStr">
         <is>
-          <t>SA14B#  ml  70.0
+          <t>SA14B  ml  70.0
 TEAVA MAT PL (PP, PE, PP-R) IMBINARE PRIN SUDURA PRIN POLIFUZIUNE, LA CTII IND, D=20 MM</t>
         </is>
       </c>
@@ -7252,7 +7252,7 @@
       </c>
       <c r="B329" s="8" t="inlineStr">
         <is>
-          <t>SA14C#  m  40.0
+          <t>SA14C  m  40.0
 TEAVA MAT PL (PP, PE, PP-R) IMBINATA PRIN SUDURA PRIN POLIFUZIUNE, LA CTII IND 25 MM DESIGN STUDIO S.R.L. - proiect inițial 424/2018 - proiect actualizat integral 424-rev/ 2024</t>
         </is>
       </c>
@@ -9057,13 +9057,13 @@
       </c>
       <c r="B416" s="8" t="inlineStr">
         <is>
-          <t>CK23A#  mp  5.0
+          <t>CK23A  mp  5.0
 Ferestre din mase plastice cu unul sau mai multe canaturi, supraf toc mai mare 1.00 mp, la ctii cu H mai mic sau egal 35 m</t>
         </is>
       </c>
       <c r="C416" s="8" t="inlineStr">
         <is>
-          <t>CK23A#  m  5.0
+          <t>CK23A  m  5.0
 Ferestre din mase plastice cu unul sau mai multe canaturi, supraf toc mai mare 1.00 mp, la ctii cu H mai mic sau egal mp material: manopera: utilaj: transport: 20.L FERESTRE DIN PROFILE PVC CU GEAM TERMOIZOLANT MP.</t>
         </is>
       </c>
@@ -9185,7 +9185,7 @@
       </c>
       <c r="B422" s="8" t="inlineStr">
         <is>
-          <t>CF15C#  mp  156.0
+          <t>CF15C  mp  156.0
 Tencuieli interioare finisaj fin sclivisite, de 0.5 cm grosime, la pereti din beton cu suprafete plane, executate manual, cu mortar DESIGN STUDIO S.R.L. - proiect inițial 424/2018 - proiect actualizat integral 424-rev/ 2024</t>
         </is>
       </c>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="B424" s="8" t="inlineStr">
         <is>
-          <t>CI06C#  mp  156.0
+          <t>CI06C  mp  156.0
 Placaj faianta, aceeasi culoare si format, 15 cm-30x30 cm, fixate cu aditiv, pe supr plane pereti si stalpi</t>
         </is>
       </c>
@@ -10076,13 +10076,13 @@
       </c>
       <c r="B465" s="8" t="inlineStr">
         <is>
-          <t>SB09A#  buc  10.0
+          <t>SB09A  buc  10.0
 PIESE LEG (COT, RED, PIESA CURAT MUFA DUBLA, COMP DILAT) PE, PP, PP-R CANAL IMB GRN CAUC DN32 MM</t>
         </is>
       </c>
       <c r="C465" s="8" t="inlineStr">
         <is>
-          <t>SB09A#    0.0
+          <t>SB09A    0.0
 PIESE LEG (COT, RED, PIESA CURAT MUFA DUBLA, COMP DILAT) PE, PP, PP-R CANAL IMB GRN CAUC</t>
         </is>
       </c>
@@ -10099,13 +10099,13 @@
       </c>
       <c r="B466" s="8" t="inlineStr">
         <is>
-          <t>SB09A#  buc  10.0
+          <t>SB09A  buc  10.0
 PIESE LEG (COT, RED, PIESA CURAT MUFA DUBLA, COMP DILAT) PE, PP, PP-R CANAL IMB GRN CAUC DN32 MM</t>
         </is>
       </c>
       <c r="C466" s="8" t="inlineStr">
         <is>
-          <t>SB09A#    0.0
+          <t>SB09A    0.0
 PIESE LEG (COT, RED, PIESA CURAT MUFA DUBLA, COMP DILAT) PE, PP, PP-R CANAL IMB GRN CAUC</t>
         </is>
       </c>
@@ -10122,13 +10122,13 @@
       </c>
       <c r="B467" s="8" t="inlineStr">
         <is>
-          <t>SB09B#  m  10.0
+          <t>SB09B  m  10.0
 PIESE LEG (COT, RED, PIESA CURAT MUFA DUBLA, COMP DILAT) PE, PP, PP-R CANAL IMB GRN CAUC DN=40 MM</t>
         </is>
       </c>
       <c r="C467" s="8" t="inlineStr">
         <is>
-          <t>SB09B#  buc  10.0
+          <t>SB09B  buc  10.0
 PIESE LEG (COT, RED, PIESA CURAT MUFA DUBLA, COMP DILAT) PE, PP, PP-R CANAL IMB GRN CAUC DN=40 MM material: manopera: utilaj: transport: 22.L COT PP 40X45 B?C.</t>
         </is>
       </c>
@@ -10166,7 +10166,7 @@
       </c>
       <c r="B469" s="8" t="inlineStr">
         <is>
-          <t>SA14B#  ml  30.0
+          <t>SA14B  ml  30.0
 TEAVA MAT PL (PP, PE, PP-R) IMBINARE PRIN SUDURA PRIN POLIFUZIUNE, LA CTII IND, D=20 MM</t>
         </is>
       </c>
@@ -10292,7 +10292,7 @@
       </c>
       <c r="B475" s="8" t="inlineStr">
         <is>
-          <t>SA14C#  m  10.0
+          <t>SA14C  m  10.0
 TEAVA MAT PL (PP, PE, PP-R) IMBINATA PRIN SUDURA PRIN POLIFUZIUNE, LA CTII IND. , D= 25 MM DESIGN STUDIO S.R.L. - proiect inițial 424/2018 - proiect actualizat integral 424-rev / 2024 =</t>
         </is>
       </c>
@@ -11561,13 +11561,13 @@
       </c>
       <c r="B536" s="8" t="inlineStr">
         <is>
-          <t>W2F03A#  buc  38.0
+          <t>W2F03A  buc  38.0
 Corp de iluminat exterior ornamental, pentru o lampa cu vapori de mercur sau sodiu montat pe stalp de metal de 5 m</t>
         </is>
       </c>
       <c r="C536" s="8" t="inlineStr">
         <is>
-          <t>W2F03A#  m  38.0
+          <t>W2F03A  m  38.0
 Corp de iluminat exterior ornamental, pentru o lampa cu vapori de mercur sau sodiu montat pe stalp de metal de buc material: manopera: utilaj: transport: 16.L Corp de iluminat stradal tip LED 50W , P= 50W, IP65,flux 4500 lumeni BUC.</t>
         </is>
       </c>
@@ -12031,7 +12031,7 @@
       </c>
       <c r="B558" s="8" t="inlineStr">
         <is>
-          <t>SF01C#  m  345.0
+          <t>SF01C  m  345.0
 EFECT PROBA ETANS PRES INSTAL APA CALDA, RECE, DIN TEAVA PVC (G) SAU PE. PP. PP-R D= 16-110 MM</t>
         </is>
       </c>
@@ -12052,7 +12052,7 @@
       </c>
       <c r="B559" s="8" t="inlineStr">
         <is>
-          <t>SF05C#  m  345.0
+          <t>SF05C  m  345.0
 SPALARE INSTAL APA RECE SAU CALDA , EXECUTATA DIN TEVI PVC (G) , PE, PP, PP-R, D= 20-75 MM</t>
         </is>
       </c>
@@ -13164,7 +13164,7 @@
       </c>
       <c r="B613" s="8" t="inlineStr">
         <is>
-          <t>RPCE29A#  mp  1256.0
+          <t>RPCE29A  mp  1256.0
 PRELATA PENTRU PROTEJAREA TERASEI PE TIMP PLOIOS PE DURATA REFACERII</t>
         </is>
       </c>
@@ -13206,7 +13206,7 @@
       </c>
       <c r="B615" s="8" t="inlineStr">
         <is>
-          <t>CK25A#  mp  7.0
+          <t>CK25A  mp  7.0
 USI PROFILURI MASE PLASTICE, 1 CANAT, SUPR. TOC MAI MIC SAU EGAL 7 MP, INC. ARMATURI SI ACCESORII, MONTATE IN ZID DE ORICE FEL LA C-TII CU H MAI MIC DE 35 M INCLUSIV</t>
         </is>
       </c>
@@ -16054,7 +16054,7 @@
       </c>
       <c r="B758" s="8" t="inlineStr">
         <is>
-          <t>IC31A1#  m  36.0
+          <t>IC31A1  m  36.0
 TEAVA DIN CUPRU MONTATA PRIN SUDURA LA LEGATURA CORPURILOR AI APARATELOR DE INSTALATIILE DE IMCALZIRE CENTRALA CU DIAMETRUL EXTERIOR DE PANA LA 15.0 MM INCLUSIV</t>
         </is>
       </c>
@@ -19325,7 +19325,7 @@
     <row r="922" ht="20" customHeight="1">
       <c r="A922" s="6" t="inlineStr">
         <is>
-          <t>Categoria de lucrari: ALIMENTARE CU E.E. SI ILUMINAT</t>
+          <t>Categoria de lucrari: CANALIZARE</t>
         </is>
       </c>
     </row>
@@ -19340,8 +19340,8 @@
       </c>
       <c r="C923" s="8" t="inlineStr">
         <is>
-          <t>W1F12D  buc  1.0
-INCERCARI PENTRU MASURAREA TENSIUNII DE ATINGERE SI DE PAS. material: manopera: utilaj: transport: procent material manopera utilaj transport total</t>
+          <t>IA37E1  buc  2.0
+REZERVOR DEPOZIT PT. COMBUSTIBIL LICHID, CILINDRIC CAPACITATE 30000 L. material: manopera: utilaj: transport: 16.L BAZIN VIDANJABIL PAFSIN 20 MC BUC. 16.L BAZIN VIDANJABIL 40 MC BUC.</t>
         </is>
       </c>
       <c r="D923" s="9" t="inlineStr">
@@ -19353,7 +19353,7 @@
     <row r="924" ht="20" customHeight="1">
       <c r="A924" s="6" t="inlineStr">
         <is>
-          <t>Categoria de lucrari: CANALIZARE</t>
+          <t>Categoria de lucrari: ALIMENTARE CU E.E. SI ILUMINAT</t>
         </is>
       </c>
     </row>
@@ -19368,8 +19368,8 @@
       </c>
       <c r="C925" s="8" t="inlineStr">
         <is>
-          <t>IA37E1  buc  2.0
-REZERVOR DEPOZIT PT. COMBUSTIBIL LICHID, CILINDRIC CAPACITATE 30000 L. material: manopera: utilaj: transport: 16.L BAZIN VIDANJABIL PAFSIN 20 MC BUC. 16.L BAZIN VIDANJABIL 40 MC BUC.</t>
+          <t>W1F12D  buc  1.0
+INCERCARI PENTRU MASURAREA TENSIUNII DE ATINGERE SI DE PAS. material: manopera: utilaj: transport: procent material manopera utilaj transport total</t>
         </is>
       </c>
       <c r="D925" s="9" t="inlineStr">

</xml_diff>